<commit_message>
Fix: escritura correcta de sesiones HDR (EQD2 1-4), columnas específicas y ajustes de cartón dosimétrico
</commit_message>
<xml_diff>
--- a/Cartón dosimétrico.xlsx
+++ b/Cartón dosimétrico.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Julieta\Desktop\Cdvh_web\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{95937E3D-F571-4A75-A5ED-D8A7584BEB12}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B01EEDBF-0A8E-4665-B294-5D177C42DC67}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{55181067-1112-4DCA-89D5-DC46FE4DA41D}"/>
   </bookViews>
@@ -177,7 +177,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="10" x14ac:knownFonts="1">
+  <fonts count="12" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -246,6 +246,18 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="5">
     <fill>
@@ -915,7 +927,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="158">
+  <cellXfs count="162">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
@@ -984,29 +996,17 @@
     <xf numFmtId="0" fontId="8" fillId="3" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="37" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="8" fillId="3" borderId="37" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
     <xf numFmtId="0" fontId="8" fillId="3" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="3" borderId="35" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="36" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -1065,211 +1065,235 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="35" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="45" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="46" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="45" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="30" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="39" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="45" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="51" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="40" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="38" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="48" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="49" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="50" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="38" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="45" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="38" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="45" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="45" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="30" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="47" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="47" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="52" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="38" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="22" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="38" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="22" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="39" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="45" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="45" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="38" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="47" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="45" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="46" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="45" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="30" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="39" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="45" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="51" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="40" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="38" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="49" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="50" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="38" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="45" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="38" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="45" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="45" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="47" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="47" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="48" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="38" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="22" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="45" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="45" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="52" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="38" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="3" borderId="38" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="3" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="3" borderId="45" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="3" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="3" borderId="39" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1715,37 +1739,37 @@
     <row r="2" spans="1:10" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="14"/>
       <c r="C2" s="1"/>
-      <c r="D2" s="148" t="s">
+      <c r="D2" s="151" t="s">
         <v>43</v>
       </c>
-      <c r="E2" s="148"/>
-      <c r="F2" s="56"/>
-      <c r="G2" s="56"/>
+      <c r="E2" s="151"/>
+      <c r="F2" s="52"/>
+      <c r="G2" s="52"/>
       <c r="I2" s="14"/>
     </row>
     <row r="3" spans="1:10" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="14"/>
       <c r="C3" s="2"/>
-      <c r="D3" s="149" t="s">
+      <c r="D3" s="152" t="s">
         <v>44</v>
       </c>
-      <c r="E3" s="149"/>
+      <c r="E3" s="152"/>
       <c r="F3" s="23"/>
-      <c r="G3" s="151" t="s">
+      <c r="G3" s="154" t="s">
         <v>42</v>
       </c>
-      <c r="H3" s="151"/>
-      <c r="I3" s="152"/>
+      <c r="H3" s="154"/>
+      <c r="I3" s="155"/>
     </row>
     <row r="4" spans="1:10" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="14"/>
       <c r="C4" s="3"/>
-      <c r="D4" s="150" t="s">
+      <c r="D4" s="153" t="s">
         <v>41</v>
       </c>
-      <c r="E4" s="150"/>
-      <c r="F4" s="150"/>
-      <c r="G4" s="150"/>
+      <c r="E4" s="153"/>
+      <c r="F4" s="153"/>
+      <c r="G4" s="153"/>
       <c r="I4" s="14"/>
     </row>
     <row r="5" spans="1:10" ht="19.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -1778,24 +1802,24 @@
       </c>
       <c r="C8" s="30"/>
       <c r="D8" s="26"/>
-      <c r="E8" s="119"/>
-      <c r="F8" s="119"/>
-      <c r="G8" s="119"/>
-      <c r="H8" s="119"/>
-      <c r="I8" s="120"/>
+      <c r="E8" s="126"/>
+      <c r="F8" s="126"/>
+      <c r="G8" s="126"/>
+      <c r="H8" s="126"/>
+      <c r="I8" s="127"/>
       <c r="J8" s="24"/>
     </row>
     <row r="9" spans="1:10" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B9" s="80" t="s">
+      <c r="B9" s="76" t="s">
         <v>2</v>
       </c>
-      <c r="C9" s="121"/>
-      <c r="D9" s="122"/>
-      <c r="E9" s="122"/>
-      <c r="F9" s="122"/>
-      <c r="G9" s="122"/>
-      <c r="H9" s="122"/>
-      <c r="I9" s="123"/>
+      <c r="C9" s="128"/>
+      <c r="D9" s="129"/>
+      <c r="E9" s="129"/>
+      <c r="F9" s="129"/>
+      <c r="G9" s="129"/>
+      <c r="H9" s="129"/>
+      <c r="I9" s="130"/>
     </row>
     <row r="10" spans="1:10" ht="22.05" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="11" spans="1:10" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -1806,78 +1830,78 @@
       <c r="F11" s="16"/>
     </row>
     <row r="12" spans="1:10" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B12" s="82" t="s">
+      <c r="B12" s="78" t="s">
         <v>5</v>
       </c>
       <c r="C12" s="27"/>
       <c r="D12" s="12"/>
-      <c r="E12" s="124" t="s">
+      <c r="E12" s="131" t="s">
         <v>40</v>
       </c>
-      <c r="F12" s="125"/>
-      <c r="G12" s="99" t="s">
+      <c r="F12" s="132"/>
+      <c r="G12" s="104" t="s">
         <v>7</v>
       </c>
-      <c r="H12" s="133"/>
-      <c r="I12" s="81" t="s">
+      <c r="H12" s="125"/>
+      <c r="I12" s="77" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="13" spans="1:10" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B13" s="83" t="s">
+      <c r="B13" s="79" t="s">
         <v>6</v>
       </c>
       <c r="C13" s="28"/>
       <c r="D13" s="12"/>
-      <c r="E13" s="126" t="s">
+      <c r="E13" s="133" t="s">
         <v>9</v>
       </c>
-      <c r="F13" s="126"/>
-      <c r="G13" s="140" t="s">
+      <c r="F13" s="133"/>
+      <c r="G13" s="139" t="s">
         <v>14</v>
       </c>
-      <c r="H13" s="141"/>
-      <c r="I13" s="57"/>
+      <c r="H13" s="140"/>
+      <c r="I13" s="53"/>
     </row>
     <row r="14" spans="1:10" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B14" s="84" t="s">
+      <c r="B14" s="80" t="s">
         <v>35</v>
       </c>
       <c r="C14" s="11"/>
       <c r="D14" s="13"/>
-      <c r="E14" s="127" t="s">
+      <c r="E14" s="134" t="s">
         <v>10</v>
       </c>
-      <c r="F14" s="128"/>
-      <c r="G14" s="142" t="s">
+      <c r="F14" s="135"/>
+      <c r="G14" s="141" t="s">
         <v>14</v>
       </c>
-      <c r="H14" s="143"/>
-      <c r="I14" s="54"/>
+      <c r="H14" s="142"/>
+      <c r="I14" s="50"/>
     </row>
     <row r="15" spans="1:10" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="D15" s="14"/>
-      <c r="E15" s="129" t="s">
+      <c r="E15" s="145" t="s">
         <v>11</v>
       </c>
-      <c r="F15" s="130"/>
-      <c r="G15" s="140" t="s">
+      <c r="F15" s="146"/>
+      <c r="G15" s="139" t="s">
         <v>14</v>
       </c>
-      <c r="H15" s="141"/>
-      <c r="I15" s="58"/>
+      <c r="H15" s="140"/>
+      <c r="I15" s="54"/>
     </row>
     <row r="16" spans="1:10" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="D16" s="14"/>
-      <c r="E16" s="131" t="s">
+      <c r="E16" s="147" t="s">
         <v>12</v>
       </c>
-      <c r="F16" s="132"/>
-      <c r="G16" s="144" t="s">
+      <c r="F16" s="148"/>
+      <c r="G16" s="143" t="s">
         <v>14</v>
       </c>
-      <c r="H16" s="145"/>
-      <c r="I16" s="55"/>
+      <c r="H16" s="144"/>
+      <c r="I16" s="51"/>
     </row>
     <row r="17" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="E17" s="20"/>
@@ -1899,168 +1923,168 @@
       <c r="C19" s="25" t="s">
         <v>23</v>
       </c>
-      <c r="D19" s="102" t="s">
+      <c r="D19" s="111" t="s">
         <v>24</v>
       </c>
-      <c r="E19" s="103"/>
-      <c r="F19" s="102" t="s">
+      <c r="E19" s="136"/>
+      <c r="F19" s="111" t="s">
         <v>25</v>
       </c>
-      <c r="G19" s="103"/>
-      <c r="H19" s="102" t="s">
+      <c r="G19" s="136"/>
+      <c r="H19" s="111" t="s">
         <v>26</v>
       </c>
-      <c r="I19" s="106"/>
+      <c r="I19" s="112"/>
     </row>
     <row r="20" spans="1:9" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B20" s="59" t="s">
+      <c r="B20" s="55" t="s">
         <v>39</v>
       </c>
-      <c r="C20" s="60"/>
-      <c r="D20" s="107"/>
-      <c r="E20" s="108"/>
-      <c r="F20" s="107"/>
-      <c r="G20" s="108"/>
-      <c r="H20" s="136"/>
-      <c r="I20" s="137"/>
+      <c r="C20" s="56"/>
+      <c r="D20" s="113"/>
+      <c r="E20" s="114"/>
+      <c r="F20" s="113"/>
+      <c r="G20" s="114"/>
+      <c r="H20" s="137"/>
+      <c r="I20" s="138"/>
     </row>
     <row r="21" spans="1:9" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B21" s="61" t="s">
+      <c r="B21" s="57" t="s">
         <v>16</v>
       </c>
-      <c r="C21" s="62"/>
-      <c r="D21" s="109"/>
-      <c r="E21" s="110"/>
-      <c r="F21" s="109"/>
-      <c r="G21" s="110"/>
-      <c r="H21" s="91"/>
-      <c r="I21" s="92"/>
+      <c r="C21" s="58"/>
+      <c r="D21" s="115"/>
+      <c r="E21" s="116"/>
+      <c r="F21" s="115"/>
+      <c r="G21" s="116"/>
+      <c r="H21" s="96"/>
+      <c r="I21" s="97"/>
     </row>
     <row r="22" spans="1:9" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A22" s="14"/>
-      <c r="B22" s="63" t="s">
+      <c r="B22" s="59" t="s">
         <v>17</v>
       </c>
-      <c r="C22" s="62"/>
-      <c r="D22" s="109"/>
-      <c r="E22" s="110"/>
-      <c r="F22" s="109"/>
-      <c r="G22" s="110"/>
-      <c r="H22" s="91"/>
-      <c r="I22" s="92"/>
+      <c r="C22" s="58"/>
+      <c r="D22" s="115"/>
+      <c r="E22" s="116"/>
+      <c r="F22" s="115"/>
+      <c r="G22" s="116"/>
+      <c r="H22" s="96"/>
+      <c r="I22" s="97"/>
     </row>
     <row r="23" spans="1:9" ht="19.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B23" s="64" t="s">
+      <c r="B23" s="60" t="s">
         <v>20</v>
       </c>
-      <c r="C23" s="65"/>
-      <c r="D23" s="111"/>
-      <c r="E23" s="112"/>
-      <c r="F23" s="111"/>
-      <c r="G23" s="112"/>
-      <c r="H23" s="93"/>
-      <c r="I23" s="94"/>
+      <c r="C23" s="61"/>
+      <c r="D23" s="107"/>
+      <c r="E23" s="108"/>
+      <c r="F23" s="107"/>
+      <c r="G23" s="108"/>
+      <c r="H23" s="98"/>
+      <c r="I23" s="99"/>
     </row>
     <row r="24" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A24" s="14"/>
       <c r="B24" s="45" t="s">
         <v>18</v>
       </c>
-      <c r="C24" s="46"/>
-      <c r="D24" s="113"/>
-      <c r="E24" s="114"/>
-      <c r="F24" s="113"/>
-      <c r="G24" s="114"/>
-      <c r="H24" s="134"/>
-      <c r="I24" s="135"/>
+      <c r="C24" s="86"/>
+      <c r="D24" s="117"/>
+      <c r="E24" s="118"/>
+      <c r="F24" s="117"/>
+      <c r="G24" s="118"/>
+      <c r="H24" s="156"/>
+      <c r="I24" s="157"/>
     </row>
     <row r="25" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A25" s="14"/>
-      <c r="B25" s="47" t="s">
+      <c r="B25" s="46" t="s">
         <v>19</v>
       </c>
-      <c r="C25" s="48"/>
-      <c r="D25" s="115"/>
-      <c r="E25" s="116"/>
-      <c r="F25" s="115"/>
-      <c r="G25" s="116"/>
-      <c r="H25" s="117"/>
-      <c r="I25" s="118"/>
+      <c r="C25" s="87"/>
+      <c r="D25" s="119"/>
+      <c r="E25" s="120"/>
+      <c r="F25" s="119"/>
+      <c r="G25" s="120"/>
+      <c r="H25" s="158"/>
+      <c r="I25" s="159"/>
     </row>
     <row r="26" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A26" s="14"/>
-      <c r="B26" s="49" t="s">
+      <c r="B26" s="47" t="s">
         <v>27</v>
       </c>
-      <c r="C26" s="50"/>
-      <c r="D26" s="85"/>
-      <c r="E26" s="86"/>
-      <c r="F26" s="85"/>
-      <c r="G26" s="86"/>
-      <c r="H26" s="117"/>
-      <c r="I26" s="118"/>
+      <c r="C26" s="88"/>
+      <c r="D26" s="121"/>
+      <c r="E26" s="122"/>
+      <c r="F26" s="121"/>
+      <c r="G26" s="122"/>
+      <c r="H26" s="158"/>
+      <c r="I26" s="159"/>
     </row>
     <row r="27" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A27" s="14"/>
-      <c r="B27" s="51" t="s">
+      <c r="B27" s="48" t="s">
         <v>28</v>
       </c>
-      <c r="C27" s="50"/>
-      <c r="D27" s="85"/>
-      <c r="E27" s="86"/>
-      <c r="F27" s="85"/>
-      <c r="G27" s="86"/>
-      <c r="H27" s="117"/>
-      <c r="I27" s="118"/>
+      <c r="C27" s="88"/>
+      <c r="D27" s="121"/>
+      <c r="E27" s="122"/>
+      <c r="F27" s="121"/>
+      <c r="G27" s="122"/>
+      <c r="H27" s="158"/>
+      <c r="I27" s="159"/>
     </row>
     <row r="28" spans="1:9" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A28" s="14"/>
-      <c r="B28" s="52" t="s">
+      <c r="B28" s="49" t="s">
         <v>29</v>
       </c>
-      <c r="C28" s="53"/>
-      <c r="D28" s="89"/>
-      <c r="E28" s="90"/>
-      <c r="F28" s="89"/>
-      <c r="G28" s="90"/>
-      <c r="H28" s="138"/>
-      <c r="I28" s="139"/>
+      <c r="C28" s="89"/>
+      <c r="D28" s="123"/>
+      <c r="E28" s="124"/>
+      <c r="F28" s="123"/>
+      <c r="G28" s="124"/>
+      <c r="H28" s="160"/>
+      <c r="I28" s="161"/>
     </row>
     <row r="29" spans="1:9" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B29" s="66" t="s">
+      <c r="B29" s="62" t="s">
         <v>21</v>
       </c>
-      <c r="C29" s="67"/>
-      <c r="D29" s="146"/>
-      <c r="E29" s="147"/>
-      <c r="F29" s="146"/>
-      <c r="G29" s="147"/>
-      <c r="H29" s="136"/>
-      <c r="I29" s="137"/>
+      <c r="C29" s="63"/>
+      <c r="D29" s="149"/>
+      <c r="E29" s="150"/>
+      <c r="F29" s="149"/>
+      <c r="G29" s="150"/>
+      <c r="H29" s="137"/>
+      <c r="I29" s="138"/>
     </row>
     <row r="30" spans="1:9" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B30" s="63" t="s">
+      <c r="B30" s="59" t="s">
         <v>3</v>
       </c>
-      <c r="C30" s="68"/>
-      <c r="D30" s="95"/>
-      <c r="E30" s="96"/>
-      <c r="F30" s="95"/>
-      <c r="G30" s="96"/>
-      <c r="H30" s="91"/>
-      <c r="I30" s="92"/>
+      <c r="C30" s="64"/>
+      <c r="D30" s="100"/>
+      <c r="E30" s="101"/>
+      <c r="F30" s="100"/>
+      <c r="G30" s="101"/>
+      <c r="H30" s="96"/>
+      <c r="I30" s="97"/>
     </row>
     <row r="31" spans="1:9" ht="19.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B31" s="69" t="s">
+      <c r="B31" s="65" t="s">
         <v>22</v>
       </c>
-      <c r="C31" s="65"/>
-      <c r="D31" s="111"/>
-      <c r="E31" s="112"/>
-      <c r="F31" s="111"/>
-      <c r="G31" s="112"/>
-      <c r="H31" s="93"/>
-      <c r="I31" s="94"/>
+      <c r="C31" s="61"/>
+      <c r="D31" s="107"/>
+      <c r="E31" s="108"/>
+      <c r="F31" s="107"/>
+      <c r="G31" s="108"/>
+      <c r="H31" s="98"/>
+      <c r="I31" s="99"/>
     </row>
     <row r="32" spans="1:9" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B32" s="21"/>
@@ -2079,87 +2103,87 @@
       <c r="C34" s="31" t="s">
         <v>34</v>
       </c>
-      <c r="D34" s="104" t="s">
+      <c r="D34" s="109" t="s">
         <v>36</v>
       </c>
-      <c r="E34" s="105"/>
-      <c r="F34" s="99" t="s">
+      <c r="E34" s="110"/>
+      <c r="F34" s="104" t="s">
         <v>37</v>
       </c>
-      <c r="G34" s="100"/>
-      <c r="H34" s="100"/>
-      <c r="I34" s="101"/>
+      <c r="G34" s="105"/>
+      <c r="H34" s="105"/>
+      <c r="I34" s="106"/>
       <c r="J34" s="24"/>
     </row>
     <row r="35" spans="2:10" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B35" s="70" t="s">
+      <c r="B35" s="66" t="s">
         <v>8</v>
       </c>
-      <c r="C35" s="71"/>
-      <c r="D35" s="95"/>
-      <c r="E35" s="96"/>
-      <c r="F35" s="72"/>
-      <c r="G35" s="153"/>
-      <c r="H35" s="73"/>
-      <c r="I35" s="74"/>
+      <c r="C35" s="67"/>
+      <c r="D35" s="100"/>
+      <c r="E35" s="101"/>
+      <c r="F35" s="68"/>
+      <c r="G35" s="81"/>
+      <c r="H35" s="69"/>
+      <c r="I35" s="70"/>
     </row>
     <row r="36" spans="2:10" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B36" s="34" t="s">
         <v>9</v>
       </c>
       <c r="C36" s="35"/>
-      <c r="D36" s="97"/>
-      <c r="E36" s="98"/>
+      <c r="D36" s="102"/>
+      <c r="E36" s="103"/>
       <c r="F36" s="36"/>
-      <c r="G36" s="154"/>
+      <c r="G36" s="82"/>
       <c r="H36" s="36"/>
       <c r="I36" s="37"/>
     </row>
     <row r="37" spans="2:10" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B37" s="70" t="s">
+      <c r="B37" s="66" t="s">
         <v>10</v>
       </c>
-      <c r="C37" s="75"/>
-      <c r="D37" s="95"/>
-      <c r="E37" s="96"/>
-      <c r="F37" s="76"/>
-      <c r="G37" s="155"/>
-      <c r="H37" s="76"/>
-      <c r="I37" s="77"/>
+      <c r="C37" s="71"/>
+      <c r="D37" s="100"/>
+      <c r="E37" s="101"/>
+      <c r="F37" s="72"/>
+      <c r="G37" s="83"/>
+      <c r="H37" s="72"/>
+      <c r="I37" s="73"/>
     </row>
     <row r="38" spans="2:10" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B38" s="38" t="s">
         <v>32</v>
       </c>
       <c r="C38" s="35"/>
-      <c r="D38" s="85"/>
-      <c r="E38" s="86"/>
+      <c r="D38" s="90"/>
+      <c r="E38" s="91"/>
       <c r="F38" s="36"/>
-      <c r="G38" s="154"/>
+      <c r="G38" s="82"/>
       <c r="H38" s="39"/>
       <c r="I38" s="37"/>
     </row>
     <row r="39" spans="2:10" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B39" s="70" t="s">
+      <c r="B39" s="66" t="s">
         <v>12</v>
       </c>
-      <c r="C39" s="71"/>
-      <c r="D39" s="87"/>
-      <c r="E39" s="88"/>
-      <c r="F39" s="76"/>
-      <c r="G39" s="156"/>
-      <c r="H39" s="78"/>
-      <c r="I39" s="79"/>
+      <c r="C39" s="67"/>
+      <c r="D39" s="92"/>
+      <c r="E39" s="93"/>
+      <c r="F39" s="72"/>
+      <c r="G39" s="84"/>
+      <c r="H39" s="74"/>
+      <c r="I39" s="75"/>
     </row>
     <row r="40" spans="2:10" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B40" s="40" t="s">
         <v>33</v>
       </c>
       <c r="C40" s="41"/>
-      <c r="D40" s="89"/>
-      <c r="E40" s="90"/>
+      <c r="D40" s="94"/>
+      <c r="E40" s="95"/>
       <c r="F40" s="42"/>
-      <c r="G40" s="157"/>
+      <c r="G40" s="85"/>
       <c r="H40" s="43"/>
       <c r="I40" s="44"/>
     </row>
@@ -2181,41 +2205,40 @@
     <mergeCell ref="F21:G21"/>
     <mergeCell ref="F22:G22"/>
     <mergeCell ref="F23:G23"/>
+    <mergeCell ref="E8:I8"/>
+    <mergeCell ref="C9:I9"/>
+    <mergeCell ref="E12:F12"/>
+    <mergeCell ref="E13:F13"/>
+    <mergeCell ref="E14:F14"/>
+    <mergeCell ref="G13:H13"/>
+    <mergeCell ref="G14:H14"/>
+    <mergeCell ref="H25:I25"/>
+    <mergeCell ref="H27:I27"/>
+    <mergeCell ref="H26:I26"/>
+    <mergeCell ref="D30:E30"/>
+    <mergeCell ref="G12:H12"/>
+    <mergeCell ref="H22:I22"/>
+    <mergeCell ref="D19:E19"/>
     <mergeCell ref="H23:I23"/>
     <mergeCell ref="H24:I24"/>
     <mergeCell ref="H29:I29"/>
     <mergeCell ref="H28:I28"/>
-    <mergeCell ref="G13:H13"/>
-    <mergeCell ref="G14:H14"/>
     <mergeCell ref="G15:H15"/>
     <mergeCell ref="G16:H16"/>
     <mergeCell ref="F24:G24"/>
     <mergeCell ref="E15:F15"/>
     <mergeCell ref="E16:F16"/>
-    <mergeCell ref="F19:G19"/>
-    <mergeCell ref="G12:H12"/>
-    <mergeCell ref="H22:I22"/>
-    <mergeCell ref="E8:I8"/>
-    <mergeCell ref="C9:I9"/>
-    <mergeCell ref="E12:F12"/>
-    <mergeCell ref="E13:F13"/>
-    <mergeCell ref="E14:F14"/>
-    <mergeCell ref="D19:E19"/>
-    <mergeCell ref="D34:E34"/>
+    <mergeCell ref="D24:E24"/>
+    <mergeCell ref="D25:E25"/>
+    <mergeCell ref="D26:E26"/>
+    <mergeCell ref="D27:E27"/>
+    <mergeCell ref="D28:E28"/>
     <mergeCell ref="H19:I19"/>
     <mergeCell ref="D20:E20"/>
     <mergeCell ref="D21:E21"/>
     <mergeCell ref="D22:E22"/>
     <mergeCell ref="D23:E23"/>
-    <mergeCell ref="D24:E24"/>
-    <mergeCell ref="D25:E25"/>
-    <mergeCell ref="D26:E26"/>
-    <mergeCell ref="D27:E27"/>
-    <mergeCell ref="D28:E28"/>
-    <mergeCell ref="H25:I25"/>
-    <mergeCell ref="H27:I27"/>
-    <mergeCell ref="H26:I26"/>
-    <mergeCell ref="D30:E30"/>
+    <mergeCell ref="F19:G19"/>
     <mergeCell ref="D38:E38"/>
     <mergeCell ref="D39:E39"/>
     <mergeCell ref="D40:E40"/>
@@ -2228,6 +2251,7 @@
     <mergeCell ref="D31:E31"/>
     <mergeCell ref="F30:G30"/>
     <mergeCell ref="F31:G31"/>
+    <mergeCell ref="D34:E34"/>
   </mergeCells>
   <printOptions horizontalCentered="1" verticalCentered="1"/>
   <pageMargins left="0.25" right="0.25" top="0.25" bottom="0.25" header="0" footer="0"/>

</xml_diff>